<commit_message>
Shorts R1 Excel: compra en metros Novaktex 4.5 y Bahía 2.7 m/kg
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORTS_R1_Plan_2200und.xlsx
+++ b/SHORTS_R1_Plan_2200und.xlsx
@@ -10,14 +10,15 @@
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
     <sheet name="Cantidades" sheetId="2" r:id="rId2"/>
     <sheet name="Compra tela adicional" sheetId="3" r:id="rId3"/>
-    <sheet name="Licra Bahía" sheetId="4" r:id="rId4"/>
+    <sheet name="Compra metros Novaktex" sheetId="4" r:id="rId4"/>
+    <sheet name="Licra Bahía" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="61">
   <si>
     <t>SHORT SPORT R1 — plan 2.200 und</t>
   </si>
@@ -67,16 +68,37 @@
     <t>Kg tela compra adicional (Negro + Gris)</t>
   </si>
   <si>
+    <t>Rendimiento Novaktex (short)</t>
+  </si>
+  <si>
+    <t>4.5 m / kg</t>
+  </si>
+  <si>
+    <t>Metros Novaktex — programa total</t>
+  </si>
+  <si>
+    <t>Metros Novaktex — compra adicional</t>
+  </si>
+  <si>
     <t>Licra Bahía — consumo</t>
   </si>
   <si>
+    <t>Rendimiento Bahía (licra)</t>
+  </si>
+  <si>
+    <t>2.7 m / kg</t>
+  </si>
+  <si>
     <t>Kg licra Bahía (2.200 und)</t>
   </si>
   <si>
+    <t>Metros licra Bahía (compra)</t>
+  </si>
+  <si>
     <t>Nota licra</t>
   </si>
   <si>
-    <t>Sin stock en archivo; considerar compra completa de licra</t>
+    <t>Sin stock en archivo; metros = compra estimada</t>
   </si>
   <si>
     <t>Unidades Shorts R1</t>
@@ -133,15 +155,39 @@
     <t>Kg compra adicional</t>
   </si>
   <si>
-    <t>Fórmula compra adicional por color:</t>
+    <t>m compra adicional</t>
+  </si>
+  <si>
+    <t>Kg compra adicional:</t>
   </si>
   <si>
     <t>max(0 ; kg Shorts − (existencia − kg Explore curvas))</t>
   </si>
   <si>
+    <t>Metros Novaktex:</t>
+  </si>
+  <si>
+    <t>kg compra × 4.5 m/kg</t>
+  </si>
+  <si>
+    <t>Compra en metros — tela Novaktex (Short R1)</t>
+  </si>
+  <si>
+    <t>Rendimiento: 4.5 m por kg</t>
+  </si>
+  <si>
+    <t>Kg programa Shorts</t>
+  </si>
+  <si>
+    <t>m programa</t>
+  </si>
+  <si>
     <t>Licra Bahía — Shorts R1</t>
   </si>
   <si>
+    <t>Rendimiento Bahía: 2.7 m por kg</t>
+  </si>
+  <si>
     <t>Concepto</t>
   </si>
   <si>
@@ -152,6 +198,9 @@
   </si>
   <si>
     <t>Kg licra total</t>
+  </si>
+  <si>
+    <t>Metros licra (compra)</t>
   </si>
 </sst>
 </file>
@@ -535,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -624,31 +673,71 @@
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1287</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B15" s="4">
+        <v>430.8596999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="4">
         <v>308.0000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>19</v>
+    <row r="20" spans="1:2">
+      <c r="A20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="4">
+        <v>831.6000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -663,32 +752,32 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3">
         <v>550</v>
@@ -702,10 +791,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3">
         <v>550</v>
@@ -719,10 +808,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C6" s="3">
         <v>550</v>
@@ -736,10 +825,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C7" s="3">
         <v>550</v>
@@ -753,7 +842,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C8" s="3">
         <v>2200</v>
@@ -769,41 +858,44 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="6" width="16.7109375" customWidth="1"/>
+    <col min="2" max="7" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="B4" s="4">
         <v>317.7556</v>
@@ -820,10 +912,13 @@
       <c r="F4" s="4">
         <v>52.03439999999998</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" s="4">
+        <v>234.1547999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B5" s="4">
         <v>280.4378</v>
@@ -840,10 +935,13 @@
       <c r="F5" s="4">
         <v>43.7122</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" s="4">
+        <v>196.7049</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E6" s="4">
         <v>286</v>
@@ -851,15 +949,24 @@
       <c r="F6" s="4">
         <v>95.74659999999997</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G6" s="4">
+        <v>430.8596999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>48</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -869,44 +976,145 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="4">
+        <v>143</v>
+      </c>
+      <c r="C6" s="4">
+        <v>643.5</v>
+      </c>
+      <c r="D6" s="4">
+        <v>52.03439999999998</v>
+      </c>
+      <c r="E6" s="4">
+        <v>234.1547999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="4">
+        <v>143</v>
+      </c>
+      <c r="C7" s="4">
+        <v>643.5</v>
+      </c>
+      <c r="D7" s="4">
+        <v>43.7122</v>
+      </c>
+      <c r="E7" s="4">
+        <v>196.7049</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="4">
+        <v>286</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1287</v>
+      </c>
+      <c r="D8" s="4">
+        <v>95.74659999999997</v>
+      </c>
+      <c r="E8" s="4">
+        <v>430.8596999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="3">
-        <v>2200</v>
+      <c r="A3" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="4">
-        <v>0.14</v>
+      <c r="A5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="4">
+        <v>58</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="4">
         <v>308.0000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="4">
+        <v>831.6000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>